<commit_message>
switch around in grp 5
</commit_message>
<xml_diff>
--- a/exam_plan.xlsx
+++ b/exam_plan.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{91FD25E7-8B89-470B-933A-E38CEF75A8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{91FD25E7-8B89-470B-933A-E38CEF75A8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{363FDD0E-5B35-432D-8D53-470767D86575}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1275,7 +1275,7 @@
         <v>5</v>
       </c>
       <c r="B30" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="C30">
         <v>25</v>
@@ -1335,7 +1335,7 @@
         <v>5</v>
       </c>
       <c r="B33" t="s">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="C33">
         <v>28</v>
@@ -1347,7 +1347,6 @@
         <v>0.66319444444444475</v>
       </c>
       <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="1:8" ht="21" x14ac:dyDescent="0.25">

</xml_diff>